<commit_message>
feat: integrate LinkedIn data (SecureVerse Founder, BioShield AI, AI Safety) and update demo documentation
</commit_message>
<xml_diff>
--- a/sample_data/exported_portfolio.xlsx
+++ b/sample_data/exported_portfolio.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Second-year B.Tech student focused on backend systems architecture, distributed computing, and multi-agent AI pipelines. I design and build complex infrastructure from the ground up—currently developing a distributed tensor-sharding network and a multi-agent communication system—prioritizing system design, integration logic, and scalable architecture.</t>
+          <t>Second-year B.Tech CSE student focused on backend systems architecture, distributed computing, and multi-agent AI pipelines. Founder of SecureVerse with a mission to build secure, human-aligned AI systems. Passionate about AI Safety, Digital Forensics, Decentralized Infrastructure, and Verifiable Zero-Trust Computation.</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-28T14:04:51.301991</t>
+          <t>2026-10-28T16:38:15.524282</t>
         </is>
       </c>
     </row>
@@ -803,13 +803,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>LLM Intent Classification &amp; Routing</t>
+          <t>AI Safety &amp; Alignment</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Prompt Engineering &amp; Chains</t>
+          <t>LLM Intent Classification &amp; Routing</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>RAG &amp; Ground Truth Verification</t>
+          <t>Prompt Engineering &amp; Chains</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Adversarial Critic Systems</t>
+          <t>RAG &amp; Ground Truth Verification</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>FastAPI</t>
+          <t>Adversarial Critic Systems</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Backend &amp; Cloud</t>
+          <t>AI &amp; Machine Learning</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1271,22 +1271,22 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>RESTful API Design</t>
+          <t>Ethical AI Systems</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Backend &amp; Cloud</t>
+          <t>AI &amp; Machine Learning</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1296,22 +1296,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Asynchronous Programming (asyncio)</t>
+          <t>Predictive Computational Modeling</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Backend &amp; Cloud</t>
+          <t>AI &amp; Machine Learning</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1321,7 +1321,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>APScheduler &amp; Task Queues</t>
+          <t>FastAPI</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1331,12 +1331,12 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Tailscale VPN &amp; Mesh Networking</t>
+          <t>RESTful API Design</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1356,12 +1356,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Redis Streams &amp; Message Passing</t>
+          <t>Asynchronous Programming (asyncio)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1381,12 +1381,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Vulnerability Research &amp; Bug Bounty</t>
+          <t>APScheduler &amp; Task Queues</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Security &amp; Systems</t>
+          <t>Backend &amp; Cloud</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1421,12 +1421,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Zero-Trust Data Flow Verification</t>
+          <t>Tailscale VPN &amp; Mesh Networking</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Security &amp; Systems</t>
+          <t>Backend &amp; Cloud</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Sandboxing &amp; Isolation (Firecracker)</t>
+          <t>Redis Streams &amp; Message Passing</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Security &amp; Systems</t>
+          <t>Backend &amp; Cloud</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1471,17 +1471,17 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Technical Architecture Documentation</t>
+          <t>Vulnerability Research &amp; Bug Bounty</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Soft Skills</t>
+          <t>Security &amp; Systems</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1496,17 +1496,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Conceptual Simplification</t>
+          <t>Digital Forensics &amp; Reverse Engineering</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Soft Skills</t>
+          <t>Security &amp; Systems</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Problem Decomposition</t>
+          <t>Zero-Trust Data Flow Verification</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Soft Skills</t>
+          <t>Security &amp; Systems</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1546,20 +1546,145 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
+          <t>Futuristic Systems Design</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Distributed Systems &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Sandboxing &amp; Isolation (Firecracker)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Security &amp; Systems</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Technical Architecture Documentation</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Soft Skills</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Expert</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Conceptual Simplification</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Soft Skills</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Expert</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Problem Decomposition</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Soft Skills</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Expert</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
           <t>Cross-Team Technical Leadership</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Soft Skills</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Advanced</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1576,7 +1701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1643,42 +1768,89 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>SecureVerse</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; Lead Architect</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Navi Mumbai, India</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Founded SecureVerse to engineer decentralized zero-trust identity verification architectures, AI safety tooling, and privacy-preserving computing systems.
+Formulated end-to-end cryptographic trust chains, automated audit mechanisms, and threat mitigation models recognized in national engineering challenges.
+Directed technology roadmap, leading proof-of-concept development and cross-functional prototype verification.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Zero-Trust Architecture, Cryptography, AI Safety, System Design, Python, Distributed Ledger</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
           <t>Independent Tutoring Practice</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Mathematics &amp; Physics Tutor (Grades 10–12)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Navi Mumbai, India</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Jun 2024</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Taught 50+ high school students, translating complex scientific, mathematical, and algorithmic concepts into clear, structured lessons.
 Developed diagnostic assessment frameworks to identify conceptual bottlenecks and tailored individual curricula to improve performance by an average of 22%.
 Honed mastery of first-principles thinking, communication clarity, and pedagogical system design.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Calculus, Mechanics, First-Principles Reasoning, Pedagogical System Design</t>
         </is>
@@ -1695,7 +1867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1904,42 +2076,89 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
+          <t>BioShield AI — Computational Biosafety &amp; Health Resilience Engine</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Lead Researcher &amp; Architect</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Python, PyTorch, Predictive Modeling, Simulation Engines, FastAPI, Docker</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Engineered predictive computational modeling pipelines for simulating pathogen transmission dynamics and evaluating countermeasure strategies in real time.
+Designed distributed simulation workers to process high-throughput biological interaction datasets with deterministic validation hooks.
+Authored biosafety compliance blueprints and zero-leakage data sandboxing mechanisms for sensitive health research data.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Event-driven asynchronous worker pool; deterministic simulation checkpointing; isolated compute sandboxes with strict egress filtering.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/bioshield-ai</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>https://rajrasal.dev/projects/bioshield</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>SecureVerse — Decentralized Zero-Trust Architecture</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Systems Architect</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Founder &amp; Systems Architect</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Python, Cryptography, Zero-Trust Architecture, Distributed Ledger, REST APIs</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Architected a decentralized identity and zero-trust verification platform engineered to prevent credential theft and unauthorized access in enterprise networks.
 Formulated the end-to-end cryptographic trust chain, policy evaluation engine, and auditable logging system.
 Awarded 3rd Place at the Deal Dome Competition for superior architectural soundness and threat mitigation design.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Mutual TLS, cryptographic assertion validation, state machine based authorization engine, zero persistent plain text secrets.</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>https://github.com/Soldier224K/secureverse</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://rajrasal.dev/projects/secureverse</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>

<commit_message>
feat: enrich portfolio DB, sheets, and resumes with full GitHub project inventory
</commit_message>
<xml_diff>
--- a/sample_data/exported_portfolio.xlsx
+++ b/sample_data/exported_portfolio.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-28T16:38:15.524282</t>
+          <t>2026-10-28T17:08:34.118779</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>TypeScript / JavaScript</t>
+          <t>Rust</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>SQL (PostgreSQL, SQLite)</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Bash / Shell Scripting</t>
+          <t>TypeScript / JavaScript</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -971,17 +971,17 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Distributed Systems Architecture</t>
+          <t>SQL (PostgreSQL, SQLite)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Distributed Systems &amp; Architecture</t>
+          <t>Languages</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -996,22 +996,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Tensor Sharding &amp; Compute Networks</t>
+          <t>Bash / Shell Scripting</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Distributed Systems &amp; Architecture</t>
+          <t>Languages</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Decoupled Orchestration</t>
+          <t>Distributed Systems Architecture</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Zero-Trust Communication Protocols</t>
+          <t>Tensor Sharding &amp; Compute Networks</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Proof-of-Compute Verification</t>
+          <t>Decoupled Orchestration</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>System Design &amp; Scalability</t>
+          <t>Zero-Trust Communication Protocols</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1121,17 +1121,17 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Multi-Agent AI Pipelines</t>
+          <t>Proof-of-Compute Verification</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>AI &amp; Machine Learning</t>
+          <t>Distributed Systems &amp; Architecture</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1146,17 +1146,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>AI Safety &amp; Alignment</t>
+          <t>System Design &amp; Scalability</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>AI &amp; Machine Learning</t>
+          <t>Distributed Systems &amp; Architecture</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1171,17 +1171,17 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>LLM Intent Classification &amp; Routing</t>
+          <t>Soroban Smart Contracts (Stellar)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>AI &amp; Machine Learning</t>
+          <t>Distributed Systems &amp; Architecture</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Prompt Engineering &amp; Chains</t>
+          <t>Multi-Agent AI Pipelines</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>RAG &amp; Ground Truth Verification</t>
+          <t>AI Safety &amp; Alignment</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Adversarial Critic Systems</t>
+          <t>LLM Intent Classification &amp; Routing</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Ethical AI Systems</t>
+          <t>Prompt Engineering &amp; Chains</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Predictive Computational Modeling</t>
+          <t>Progressive RAG &amp; Memory Layers</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Intermediate</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1321,17 +1321,17 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>FastAPI</t>
+          <t>Adversarial Critic Systems</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Backend &amp; Cloud</t>
+          <t>AI &amp; Machine Learning</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1346,22 +1346,22 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>RESTful API Design</t>
+          <t>Ethical AI Systems</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Backend &amp; Cloud</t>
+          <t>AI &amp; Machine Learning</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1371,22 +1371,22 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Asynchronous Programming (asyncio)</t>
+          <t>Predictive Computational Modeling</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Backend &amp; Cloud</t>
+          <t>AI &amp; Machine Learning</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Intermediate</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>APScheduler &amp; Task Queues</t>
+          <t>FastAPI</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1406,12 +1406,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Tailscale VPN &amp; Mesh Networking</t>
+          <t>RESTful API Design</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1431,12 +1431,12 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Redis Streams &amp; Message Passing</t>
+          <t>Asynchronous Programming (asyncio)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1456,12 +1456,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Advanced</t>
+          <t>Expert</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -1471,12 +1471,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Vulnerability Research &amp; Bug Bounty</t>
+          <t>AWS Lambda &amp; Serverless Pipelines</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Security &amp; Systems</t>
+          <t>Backend &amp; Cloud</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1496,12 +1496,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Digital Forensics &amp; Reverse Engineering</t>
+          <t>MongoDB &amp; Aggregation Framework</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Security &amp; Systems</t>
+          <t>Backend &amp; Cloud</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1521,12 +1521,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Zero-Trust Data Flow Verification</t>
+          <t>APScheduler &amp; Task Queues</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Security &amp; Systems</t>
+          <t>Backend &amp; Cloud</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1546,12 +1546,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Futuristic Systems Design</t>
+          <t>Tailscale VPN &amp; Mesh Networking</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Distributed Systems &amp; Architecture</t>
+          <t>Backend &amp; Cloud</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1571,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Sandboxing &amp; Isolation (Firecracker)</t>
+          <t>Redis Streams &amp; Message Passing</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Security &amp; Systems</t>
+          <t>Backend &amp; Cloud</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1596,17 +1596,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Technical Architecture Documentation</t>
+          <t>Vulnerability Research &amp; Bug Bounty</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Soft Skills</t>
+          <t>Security &amp; Systems</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1621,17 +1621,17 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Conceptual Simplification</t>
+          <t>Digital Forensics &amp; Reverse Engineering</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Soft Skills</t>
+          <t>Security &amp; Systems</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -1646,17 +1646,17 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Problem Decomposition</t>
+          <t>Zero-Trust Data Flow Verification</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Soft Skills</t>
+          <t>Security &amp; Systems</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Expert</t>
+          <t>Advanced</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1671,20 +1671,170 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
+          <t>Futuristic Systems Design</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Distributed Systems &amp; Architecture</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Non-STL Algorithm Engineering</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Security &amp; Systems</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Sandboxing &amp; Isolation (Firecracker)</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Security &amp; Systems</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Technical Architecture Documentation</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Soft Skills</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Expert</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Conceptual Simplification</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Soft Skills</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Expert</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Problem Decomposition</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Soft Skills</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Expert</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
           <t>Cross-Team Technical Leadership</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>Soft Skills</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Advanced</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1867,7 +2017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1877,7 +2027,7 @@
     <col width="54" customWidth="1" min="5" max="5"/>
     <col width="54" customWidth="1" min="6" max="6"/>
     <col width="54" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="54" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -2161,6 +2311,288 @@
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive Diplomat — Multi-Agent Negotiation Predictor &amp; RAG</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Lead AI Systems Architect</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>TypeScript, Express, Ollama LLM, Progressive RAG, In-Memory LRU Cache, Vector-Keyword Hybrid Retrieval</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Engineered a high-performance negotiation next-turn prediction engine orchestrating a 3-persona parallel agent fan-out via Promise.all.
+Implemented a progressive RAG layer over tactical negotiation playbooks with keyword-hybrid retrieval and LRU-bounded memory.
+Enforced deterministic synthesis using temperature=0 and fixed seed assertions with strict confidence score clamping.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Parallel agent fan-out; deterministic LLM synthesis; 500-entry LRU per-request memory cache; full requirement traceability matrix.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/TypeScript-prediction-API-with-parallel-agents-and-RAG</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>https://loom.com/share/b5c92f183d2a456191b24e931168923a</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Topcoder AI Profile Video Pipeline — Async Cloud-Native Engine</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Cloud &amp; AI Pipeline Architect</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Python, AWS Lambda, MoviePy/FFmpeg, Streamlit, Asynchronous Orchestration, Docker, Render</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Architected an event-driven serverless video processing pipeline that automatically converts raw member intro footage into professional branded Topcoder videos.
+Built an AWS Lambda queue consumer for scalable background transcription, caption overlay, and audio normalization.
+Delivered an interactive Streamlit operational dashboard for cost, performance, and compute budget analysis.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Decoupled queue-driven serverless architecture; dynamic FFmpeg rendering pipeline; budget and resource observability dashboard.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/Topcoder-Profile-Intro-Video-Generator-AI-Pipeline-Async-Scalable-</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>https://topcoder-video-pipeline.onrender.com</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>DealVault &amp; Pactum — Stellar Soroban Smart Contract Escrow</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Smart Contract &amp; Backend Engineer</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Rust, Soroban Smart Contracts, Stellar Testnet, TypeScript, Express, Web3</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Co-developed an enterprise-grade escrow infrastructure and recurring commitment registry on the Stellar blockchain.
+Authored Soroban smart contracts enforcing programmatic fund locking, milestone verification, and automated payouts.
+Constructed a tamper-proof on-chain compliance history tracking fulfillment status for service-level commitments.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Non-custodial smart contract vaults; state-machine commitment tracker; cryptographic transaction signing via Stellar SDK.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/dealvault-platform-escrow</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/Pactum</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>DSA SpaceOPs — Satellite Mission Operations &amp; Navigation Engine</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Systems &amp; Algorithm Engineer</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>C++, Non-STL Custom Data Structures, AVL Trees, Priority Queues, Graph Algorithms, Dijkstra</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Engineered a mission control and cislunar spacecraft communications router implementing 7 custom data structures completely from scratch without STL containers.
+Implemented an AVL self-balancing mission registry, Dijkstra minimum-latency routing for cislunar mesh networks, and priority queue activity arbiters.
+Designed an abort-sequence navigational rollback stack with zero memory leaks and deterministic sub-millisecond execution.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Zero-STL core architecture; custom self-balancing AVL trees; Dijkstra shortest-path network topology; O(1) abort stack rollback.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/DSA-SpaceOPs</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/DSA-SpaceOPs</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Exam Question Paper Generator — ITM Skills University</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Desktop Software Architect</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Java, Swing MVC, Custom Graphics2D, File I/O Streams, Deterministic Paper Synthesis</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Engineered a database-less desktop Java application for faculty at ITM Skills University and School of Future Tech.
+Built an algorithmic question selector that generates balanced examination papers adhering to difficulty, topic weights, and mark constraints.
+Authored complete institutional software documentation and mathematical generation proofs.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Zero-database portability using native file streams; pure MVC architecture; custom Graphics2D print formatting.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/ExamQuestionPaperGenerator_JAVA</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/ExamQuestionPaperGenerator_JAVA/blob/main/ExamQuestionPaperGeneratorDocumentation.pdf</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>WorkHub — Coworking Space Management Platform</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Backend &amp; Database Architect</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Node.js, Express, MongoDB, Aggregation Pipeline, JWT RBAC, QR Code Verification</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Engineered a coworking space reservation backend featuring zero-double-booking atomic concurrency.
+Implemented real-time availability scrubbing and MongoDB aggregation pipelines for space utilization analytics.
+Built dynamic floorplan coordinate mapping and QR-based automated desk unlock verification.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Atomic reservation locking; 2D floorplan coordinate management; multi-role JWT RBAC security.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/WorkHub</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/Soldier224K/WorkHub</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>